<commit_message>
Add second opportunity link
</commit_message>
<xml_diff>
--- a/Pinktabletrackerlocal.xlsx
+++ b/Pinktabletrackerlocal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/julianestrada/Downloads/interactivetablemap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22344427-D1AF-8147-96A1-6B89E9427385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701F02A1-B03B-9D4B-B920-583079AE70D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4060" yWindow="3160" windowWidth="27240" windowHeight="16440" xr2:uid="{FD50FAA3-49BA-8240-9E13-4B4D6922A4C0}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
   </externalReferences>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="697">
   <si>
     <t>Household Name</t>
   </si>
@@ -2128,6 +2128,9 @@
   </si>
   <si>
     <t>https://curebound.lightning.force.com/lightning/r/Opportunity/006QU00000lQkx0YAC/view</t>
+  </si>
+  <si>
+    <t>https://curebound.lightning.force.com/lightning/r/Opportunity/006QU00000qehEnYAI/view</t>
   </si>
 </sst>
 </file>
@@ -8168,8 +8171,7 @@
     <col min="3" max="3" width="24.6640625" customWidth="1"/>
     <col min="4" max="4" width="22.1640625" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
-    <col min="6" max="6" width="84.33203125" customWidth="1"/>
-    <col min="7" max="7" width="45" customWidth="1"/>
+    <col min="6" max="7" width="84.33203125" customWidth="1"/>
     <col min="8" max="8" width="47.83203125" customWidth="1"/>
     <col min="9" max="9" width="47" customWidth="1"/>
   </cols>
@@ -8661,6 +8663,9 @@
       </c>
       <c r="F27" t="s">
         <v>117</v>
+      </c>
+      <c r="G27" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update local seating data
</commit_message>
<xml_diff>
--- a/Pinktabletrackerlocal.xlsx
+++ b/Pinktabletrackerlocal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/julianestrada/Downloads/interactivetablemap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66138E5-61B7-7744-A7AA-F866E6D5D88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D33769E8-74A5-224E-8449-7C5B67869E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-34820" yWindow="2020" windowWidth="27240" windowHeight="16440" xr2:uid="{FD50FAA3-49BA-8240-9E13-4B4D6922A4C0}"/>
   </bookViews>
@@ -3045,7 +3045,7 @@
     <t xml:space="preserve">Issue tickets to Michelle Kim at Michellekim2020@yahoo.com </t>
   </si>
   <si>
-    <t>Polamalu Concert 2026 Tickets | Opportunity | Salesforce</t>
+    <t>https://curebound.lightning.force.com/lightning/r/Opportunity/006QU00000u2DFRYA2/view</t>
   </si>
 </sst>
 </file>
@@ -8344,7 +8344,7 @@
     <hyperlink ref="F133" r:id="rId9" xr:uid="{8BFBED8D-BE27-AA4B-B2E7-08315E64B68C}"/>
     <hyperlink ref="F148" r:id="rId10" display="https://curebound.lightning.force.com/lightning/r/Opportunity/006QU00000s98yXYAQ/view" xr:uid="{BF94BAB4-0CE7-E645-BAD9-0BCA6B291B73}"/>
     <hyperlink ref="G168" r:id="rId11" xr:uid="{6825F257-D41A-114A-88F7-20C2B22CF9C5}"/>
-    <hyperlink ref="F226" r:id="rId12" display="https://curebound.lightning.force.com/lightning/r/Opportunity/006QU00000u2DFRYA2/view" xr:uid="{F13A9300-ADB7-514D-9AB4-BDE540A31E7A}"/>
+    <hyperlink ref="F226" r:id="rId12" xr:uid="{F13A9300-ADB7-514D-9AB4-BDE540A31E7A}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>